<commit_message>
edit skill generate testcase based on BDD/AAS
</commit_message>
<xml_diff>
--- a/result-testcase/Test_Cases_Meta_New_Pricing_2026.xlsx
+++ b/result-testcase/Test_Cases_Meta_New_Pricing_2026.xlsx
@@ -33,7 +33,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="9.5"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,11 +78,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -455,8 +455,8 @@
   <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
@@ -464,7 +464,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
     <col width="55" customWidth="1" min="13" max="13"/>
@@ -560,7 +560,7 @@
           <t>PRICING_MGMT</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>API-PRIC-BASE-POS-001</t>
         </is>
@@ -572,13 +572,13 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Memastikan Biz Ops Admin dapat memperbarui base price pesan Meta per kategori (Marketing, Utility, Auth, Service) X negara tujuan dengan effective_at</t>
+          <t>Memastikan Biz Ops Admin dapat memperbarui base price pesan Meta per kategori (Marketing, Utility, Auth, Service) X negara tujuan dengan effective_at UTC</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1. Akses database / internal API pricing aktif.
-2. Parameter category dan country valid.</t>
+          <t>1. Akses internal API endpoint pricing aktif.
+2. Parameter category ('SERVICE') dan country ('ID') valid.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -606,16 +606,15 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim request update base price untuk category='SERVICE', country='ID', base_price=300, effective_at='2026-10-01 00:00:00 UTC'.
-2. Query tabel `meta_base_prices`.
-3. Periksa kolom effective_at.</t>
+          <t>1. [Arrange] Siapkan payload JSON update base price: {"category": "SERVICE", "country": "ID", "base_price": 300, "effective_at": "2026-10-01T00:00:00Z"}.
+2. [Act] Kirim request POST /api/v1/admin/pricing/base dengan header Authorization: Bearer &lt;bizops_token&gt;.
+3. [Assert] Query tabel meta_base_prices untuk memvalidasi persistensi data.</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>1. [API] Response merespons 200 OK dengan payload update sukses.
-2. [DB] Record tersimpan dengan base_price=300 dan status 'ACTIVE'.
-3. [DB] effective_at tersimpan sesuai timestamp UTC.</t>
+          <t>1. [API] Response merespons HTTP 200 OK dengan payload {"status": "SUCCESS", "updated_rows": 1, "data": {"category": "SERVICE", "country": "ID", "base_price": 300, "effective_at": "2026-10-01T00:00:00Z"}}.
+2. [DB] Record tersimpan di tabel meta_base_prices dengan base_price = 300, status 'ACTIVE', dan effective_at tersimpan sesuai timestamp UTC.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -640,7 +639,7 @@
           <t>PRICING_MGMT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>API-PRIC-GEN-POS-002</t>
         </is>
@@ -652,13 +651,13 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Memastikan penentuan markup general per kategori X negara berlaku untuk seluruh user tanpa custom price</t>
+          <t>Memastikan penentuan markup general per kategori X negara berlaku untuk seluruh merchant tanpa custom price</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>1. Data Base Price Meta sudah ada di DB.
-2. Akun merchant umum tidak memiliki custom markup.</t>
+          <t>1. Base Price Meta SERVICE = Rp 300 sudah aktif di DB.
+2. Akun merchant USR-STD-001 tidak memiliki custom markup.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -686,16 +685,15 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>1. Update general markup category='SERVICE', country='ID', markup_price=150, effective_at='2026-10-01 00:00:00 UTC'.
-2. Hit API estimasi biaya pesan untuk user general.
-3. Verifikasi total tarif pesan.</t>
+          <t>1. [Arrange] Siapkan payload general markup: {"category": "SERVICE", "country": "ID", "markup_price": 150, "effective_at": "2026-10-01T00:00:00Z"}.
+2. [Act] Kirim request POST /api/v1/admin/pricing/general dan request POST /api/v1/messages/estimate-rate untuk user USR-STD-001.
+3. [Assert] Verifikasi perhitungan tarif pesan dan persistensi record.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>1. [API] General markup tersimpan di tabel `general_markups`.
-2. [API] Estimasi tarif pesan = Base Price (300) + Markup (150) = Rp 450 (bulat ke atas).
-3. [DB] Audit log mencatat konfigurasi general markup.</t>
+          <t>1. [API] Endpoint estimate-rate merespons HTTP 200 OK dengan {"category": "SERVICE", "base_price": 300, "markup_price": 150, "final_rate": 450, "pricing_source": "GENERAL"}.
+2. [DB] Record tersimpan di tabel general_markups dan audit_logs mencatat event SET_GENERAL_MARKUP.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -720,7 +718,7 @@
           <t>PRICING_MGMT</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>API-PRIC-CUST-POS-003</t>
         </is>
@@ -732,13 +730,13 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Memastikan user ID tertentu dengan custom markup mendapatkan harga khusus yang mengabaikan general markup</t>
+          <t>Memastikan hierarki harga memprioritaskan custom markup merchant di atas general markup</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1. General markup = Rp 150.
-2. Custom markup untuk user_id='USR-VIP-001' diset = Rp 100.</t>
+          <t>1. General markup MARKETING = Rp 250, Base Price = Rp 650.
+2. User USR-VIP-001 memiliki custom markup MARKETING = Rp 100.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -766,16 +764,15 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim pesan dari akun 'USR-VIP-001'.
-2. Cek nilai pemotongan saldo / isolasi kredit.
-3. Bandingkan dengan user reguler 'USR-REG-002'.</t>
+          <t>1. [Arrange] Pastikan user USR-VIP-001 memiliki custom markup Rp 100 dan user umum USR-STD-001 menggunakan general markup Rp 250.
+2. [Act] Kirim request POST /api/v1/messages/estimate-rate dengan payload {"user_id": "USR-VIP-001", "category": "MARKETING", "country": "ID"}.
+3. [Assert] Verifikasi response kalkulasi tarif dan sumber harga yang diterapkan.</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>1. [API] Tarif USR-VIP-001 = Rp 300 + Rp 100 = Rp 400.
-2. [API] Tarif USR-REG-002 = Rp 300 + Rp 150 = Rp 450.
-3. [DB] Custom markup memprioritaskan override general markup 100%.</t>
+          <t>1. [API] Response merespons HTTP 200 OK dengan {"base_price": 650, "markup_price": 100, "final_rate": 750, "pricing_source": "CUSTOM", "applied_user_id": "USR-VIP-001"}.
+2. [DB] Query pricing engine mengembalikan custom record dari user_custom_markups dan tidak melakukan fallback ke general_markups.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -800,30 +797,30 @@
           <t>PRICING_MGMT</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>API-PRIC-DATE-BVA-004</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>API-PRIC-TIME-BVA-004</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Boundary Test: Penegakan tanggal efektif (effective_at) pada pricing</t>
+          <t>Verifikasi Boundary Timestamp Pergantian Harga (Relative Timestamp Seeding)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Memastikan harga baru belum berlaku sebelum timestamp effective_at tercapai</t>
+          <t>Memastikan aktivasi harga baru berlaku presisi sesuai timestamp UTC menggunakan teknik time-shift seeding</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>1. Harga lama = Rp 400.
-2. Harga baru = Rp 500 dengan effective_at='2026-10-01 00:00:00 UTC'.</t>
+          <t>1. Akses DB untuk seeding fixture pricing.
+2. Record A (Old Rate = 300) dan Record B (New Rate = 400).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -842,20 +839,21 @@
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim pesan pada waktu T-1 detik (2026-09-30 23:59:59 UTC).
-2. Kirim pesan pada waktu T (2026-10-01 00:00:00 UTC).
-3. Verifikasi pemotongan saldo pada kedua transaksi.</t>
+          <t>1. [Arrange] Seed Record A (base_price = 300, effective_at = now() - 10 days) dan Record B (base_price = 400, effective_at = now() + 1 hour).
+2. [Act - Step 1] Request POST /api/v1/messages/estimate-rate sebelum boundary transition.
+3. [Act - Step 2] Update relative timestamp Record B menjadi effective_at = now() - 1 minute (simulasi pasca boundary transition) dan request estimate-rate ulang.
+4. [Assert] Evaluasi tarif pada kedua pemanggilan.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>1. [DB] Transaksi T-1 dipotong tarif lama (Rp 400).
-2. [DB] Transaksi T dipotong tarif baru (Rp 500).
-3. [UI] Log mutasi saldo mencatat tarif yang tepat per masing-masing timestamp.</t>
+          <t>1. [API - Step 1] HTTP 200 OK dengan final_rate = 300 (pricing_version: 'OLD_RATE').
+2. [API - Step 2] HTTP 200 OK dengan final_rate = 400 (pricing_version: 'NEW_RATE').
+3. [DB] Query SELECT * FROM meta_base_prices WHERE effective_at &lt;= NOW() ORDER BY effective_at DESC LIMIT 1 mengambil Record B secara deterministik.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -865,7 +863,7 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-01: Pricing Effective Date (Covers: AC-1, AC-2, AC-3)</t>
+          <t>[Priority: Critical] US-01: Pricing Configuration &amp; Activation (Covers: AC-4)</t>
         </is>
       </c>
     </row>
@@ -880,24 +878,24 @@
           <t>PRICING_MGMT</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>API-PRIC-AUDT-POS-005</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>API-PRIC-RND-POS-005</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi pencatatan Audit Log saat terjadi perubahan harga</t>
+          <t>Verifikasi pembulatan harga ke atas (Ceil Rounding) mata uang IDR</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Memastikan sistem mencatat detail aktor, harga baru, kategori, negara, user ID, dan timestamp perubahan harga</t>
+          <t>Memastikan semua hasil kalkulasi tarif desimal dibulatkan ke bilangan bulat terdekat ke atas dalam mata uang IDR</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1. Biz Ops Admin melakukan update data harga via backend API.</t>
+          <t>1. Base price desimal = Rp 320,50 dan markup = Rp 79,25 (Total raw = Rp 399,75).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -907,7 +905,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -917,22 +915,23 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Audit, Security</t>
+          <t>Pricing, Currency</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>1. Eksekusi update harga custom untuk user_id='USR-123'.
-2. Query tabel `pricing_change_logs`.</t>
+          <t>1. [Arrange] Set konfigurasi pricing dengan komponen desimal: Base Price = 320.50, Markup = 79.25.
+2. [Act] Kirim request POST /api/v1/messages/estimate-rate untuk kalkulasi tarif per broadcast IDR.
+3. [Assert] Verifikasi nilai output kalkulasi dan tipe data amount.</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>1. [DB] Record log terbentuk dengan kolom lengkap: actor_id, new_price, category, country, user_id, valid_from.
-2. [DB] Timestamp log akurat sesuai waktu modifikasi UTC.</t>
+          <t>1. [API] Response HTTP 200 OK menghasilkan {"raw_rate": 399.75, "final_rate": 400, "currency": "IDR", "rounding_mode": "CEIL"}.
+2. [DB] Nilai yang dipotong pada payment ledger adalah integer 400 tanpa angka pecahan desimal.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -942,7 +941,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-01: Price Change Audit Logging (Covers: AC-4)</t>
+          <t>[Priority: High] US-01: Pricing Currency &amp; Rounding (Covers: AC-5)</t>
         </is>
       </c>
     </row>
@@ -954,33 +953,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>DELIVERY_CREDIT</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>WEB-BRD-FEP-POS-006</t>
+          <t>PRICING_MGMT</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JOB-PRIC-AUDT-POS-006</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi pengiriman pesan dalam Free Entry Point (FEP) Window tidak memotong kredit</t>
+          <t>Verifikasi sinkronisasi perubahan harga dan pencatatan audit log</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Memastikan pesan Marketing, Utility, Auth, dan Service yang dikirim dalam window FEP aktif (inbound CTWA/WTWA) berbiaya Rp 0</t>
+          <t>Memastikan batch update tarif oleh Biz Ops Admin tercatat lengkap pada audit log sistem</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>1. Customer melakukan inbound chat via CTWA ad.
-2. Sesi FEP Window aktif pada room percakapan.</t>
+          <t>1. Sesi Biz Ops Admin ADMIN-OPS-007 aktif.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -995,26 +993,23 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>P1-Core, FEP</t>
+          <t>Audit, Regression</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>1. Buka Chatroom pelanggan dengan flag FEP aktif.
-2. Kirim pesan template Marketing.
-3. Kirim pesan Service.
-4. Cek saldo utama WhatsApp Credit.</t>
+          <t>1. [Arrange] Siapkan batch payload pembaruan 4 kategori tarif pesan oleh ADMIN-OPS-007.
+2. [Act] Eksekusi endpoint batch POST /api/v1/admin/pricing/batch-update.
+3. [Assert] Query tabel pricing_audit_logs.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Pesan terkirim sukses tanpa loading isolasi kredit.
-2. [API] Request kirim pesan menyertakan flag `is_fep=true`.
-3. [DB] Tidak ada record pemotongan saldo / mutasi kredit (Biaya Rp 0).
-4. [UI] Saldo kredit akun tetap tidak berkurang.</t>
+          <t>1. [API] Endpoint merespons HTTP 200 OK dengan {"status": "SUCCESS", "processed_items": 4}.
+2. [DB] Tabel pricing_audit_logs mencatat 4 baris baru dengan detail actor_id = 'ADMIN-OPS-007', previous_price, new_price, action = 'UPDATE_BASE_PRICE', dan timestamp UTC.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1024,7 +1019,7 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-02: Free Entry Point Window (Covers: AC-1)</t>
+          <t>[Priority: Normal] US-01: Audit Log Configuration (Covers: AC-6)</t>
         </is>
       </c>
     </row>
@@ -1036,28 +1031,29 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>DELIVERY_CREDIT</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>JOB-BRD-ISOL-POS-007</t>
+          <t>BROADCAST_EXEC</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>WEB-BRD-ISOL-POS-007</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi Credit Isolation saat broadcast dijadwalkan dan dieksekusi</t>
+          <t>Verifikasi pembuatan broadcast dengan deduksi saldo nominal dan isolasi pesan</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Memastikan saldo kredit diisolasi (temporary deduct) sebesar (Base Price + Margin) per recipient saat jadwal tiba</t>
+          <t>Memastikan merchant dapat membuat broadcast 100 nomor melalui Multi-step Wizard, saldo terkunci presisi Rp 75.000, dan status pesan terisolasi per recipient</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>1. Saldo utama = Rp 100.000.
-2. Target broadcast = 100 nomor (tarif Rp 450/pesan, total Rp 45.000).</t>
+          <t>1. User login sebagai Merchant Admin dengan saldo awal Rp 1.000.000.
+2. Berada di dashboard broadcast /broadcast/list.
+3. File CSV contacts_100.csv (100 nomor valid) tersedia.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1077,26 +1073,28 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>P1-Core, Broadcast</t>
+          <t>P1-Core, E2E, Smoke</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>1. Buat jadwal broadcast untuk 100 nomor pada jam T.
-2. Saat jam T tiba, amati status pemotongan saldo.
-3. Periksa tabel `credit_isolations`.
-4. Tunggu delivery receipt dari Meta.</t>
+          <t>1. [Given] User berada di /broadcast/list dengan saldo Rp 1.000.000.
+2. [When - Step 1] Klik [+ Buat Broadcast Baru] (#btn-create-broadcast).
+3. [When - Step 2] Pada Wizard Step 1, pilih template 'Promo Diskon Gajian' (Kategori: MARKETING, Rp 750/pesan).
+4. [When - Step 3] Pada Wizard Step 2, upload CSV contacts_100.csv (100 penerima).
+5. [When - Step 4] Pada Wizard Step 3, pilih opsi radio 'Kirim Sekarang'.
+6. [When - Step 5] Pada Wizard Step 4 (Review), periksa ringkasan 'Total Estimasi: Rp 75.000' lalu klik [Kirim Broadcast] (#btn-submit-broadcast) dan konfirmasi modal [Ya, Eksekusi].</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Status campaign berubah menjadi 'Processing'.
-2. [DB] Saldo terisolasi sebesar Rp 45.000 (sisa saldo aktif Rp 55.000).
-3. [DB] 100 record isolasi terbentuk dengan status 'ISOLATED'.
-4. [API] Request outbound dikirim ke Meta API.</t>
+          <t>1. [Then - UI] Modal tertutup, muncul toast alert hijau: 'Broadcast berhasil dibuat dan sedang diproses', dan tabel menampilkan baris baru dengan badge [Processing].
+2. [Then - UI] Widget saldo di header terpotong real-time dari Rp 1.000.000 menjadi Rp 925.000.
+3. [And - API] POST /api/v1/broadcasts merespons HTTP 201 Created dengan {"broadcast_id": "BRD-9001", "total_contacts": 100, "locked_credits": 75000, "status": "PROCESSING"}.
+4. [And - DB] Saldo di tabel wallets berkurang Rp 75.000 dan tercatat 100 record di broadcast_recipients dengan status 'LOCKED'.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1106,7 +1104,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-02: Credit Isolation (Covers: AC-2)</t>
+          <t>[Priority: Critical] US-02: Broadcast Execution &amp; Credit Isolation (Covers: AC-1, AC-2)</t>
         </is>
       </c>
     </row>
@@ -1118,28 +1116,28 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DELIVERY_CREDIT</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+          <t>BROADCAST_EXEC</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>WEB-BRD-PART-NEG-008</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi penanganan broadcast saat saldo parsial (hanya cukup untuk sebagian target)</t>
+          <t>Verifikasi penanganan broadcast saat saldo tidak mencukupi untuk seluruh penerima</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Memastikan sistem mengirim pesan sesuai sisa saldo yang ada (FIFO) dan menggagalkan nomor sisanya dengan status saldo tidak cukup</t>
+          <t>Memastikan sistem memblokir submit broadcast di Wizard Step 4 jika total kebutuhan saldo melebihi saldo aktif merchant</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>1. Sisa saldo utama = Rp 27.000.
-2. Target broadcast = 100 nomor @ Rp 450 (kebutuhan Rp 45.000).</t>
+          <t>1. User login dengan saldo Rp 30.000 (hanya cukup untuk 40 pesan @ Rp 750).
+2. Berada di form wizard /broadcast/create.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1159,7 +1157,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Broadcast, Resiliency</t>
+          <t>Validation, UI</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -1167,18 +1165,18 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>1. Eksekusi pengiriman broadcast 100 nomor.
-2. Amati proses isolasi dan pengiriman.
-3. Periksa detail log pengiriman per nomor penerima.
-4. Cek sisa saldo akhir.</t>
+          <t>1. [Given] User berada di wizard /broadcast/create dengan saldo Rp 30.000.
+2. [When - Step 1] Pilih template MARKETING (@ Rp 750).
+3. [When - Step 2] Upload CSV contacts_100.csv (100 penerima, kebutuhan biaya = Rp 75.000).
+4. [When - Step 3] Klik [Lanjut ke Review].</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>1. [DB] Sistem mengisolasi dan mengirim 60 pesan (60 x Rp 450 = Rp 27.000).
-2. [DB] 40 nomor sisanya berstatus 'FAILED_INSUFFICIENT_BALANCE'.
-3. [UI] Dashboard Broadcast menampilkan status: 'Completed (60 Sent, 40 Failed - Saldo Kurang)'.
-4. [DB] Saldo utama menjadi Rp 0 dan tidak bernilai minus.</t>
+          <t>1. [Then - UI] Wizard terkunci di Step Review dengan error banner merah: 'Saldo kredit tidak mencukupi. Dibutuhkan Rp 75.000, saldo Anda Rp 30.000'.
+2. [Then - UI] Tombol CTA [Kirim Broadcast] berstatus disabled dan muncul CTA sekunder [Top Up Saldo].
+3. [And - API] POST /api/v1/broadcasts/validate merespons HTTP 422 Unprocessable Entity dengan error code 'INSUFFICIENT_CREDITS'.
+4. [And - DB] Saldo di tabel wallets tetap utuh Rp 30.000 tanpa mutasi.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1188,7 +1186,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-02: Partial Balance Broadcast Handling (Covers: AC-2)</t>
+          <t>[Priority: High] US-02: Insufficient Balance Handling (Covers: AC-3)</t>
         </is>
       </c>
     </row>
@@ -1200,28 +1198,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DELIVERY_CREDIT</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+          <t>ROLLBACK_MGMT</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>API-ROLL-FAIL-POS-009</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi otomatis Credit Rollback saat menerima status Failed dari Meta</t>
+          <t>Verifikasi refund saldo saat menerima webhook status Failed dari Meta</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Memastikan saldo kredit yang terisolasi langsung di-refund penuh saat Meta mengirimkan sinyal failed</t>
+          <t>Memastikan kredit per pesan otomatis di-refund kembali ke saldo merchant seketika webhook status 'failed' diterima dari Meta</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>1. Pesan telah terisolasi Rp 450.
-2. Webhook Meta mengembalikan status failed (error code 131026 / receiver unreachable).</t>
+          <t>1. Pesan broadcast MSG-BC-8801 berstatus 'SENT', saldo terpotong Rp 750, wamid = 'wamid.HBgL12345'.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1241,7 +1238,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>P1-Core, Rollback</t>
+          <t>P1-Core, Webhook</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -1249,17 +1246,16 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim webhook status 'failed' dari Meta untuk message_id='MSG-999'.
-2. Cek mutasi saldo pada tabel `credit_transactions`.
-3. Periksa saldo utama akun.</t>
+          <t>1. [Arrange] Siapkan payload webhook WhatsApp failed: {"object": "whatsapp_business_account", "entry": [{"changes": [{"value": {"statuses": [{"id": "wamid.HBgL12345", "status": "failed", "timestamp": "1726050000", "recipient_id": "6281299990001", "errors": [{"code": 131026, "title": "Message undeliverable"}]}]}}]}]}.
+2. [Act] Kirim request internal webhook POST /api/v1/webhooks/whatsapp dengan payload tersebut.
+3. [Assert] Query API mutasi saldo dan status pesan.</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>1. [API] Webhook handler memproses event failed dan merespons 200 OK.
-2. [DB] Status isolasi berubah menjadi 'ROLLED_BACK'.
-3. [DB] Saldo akun bertambah kembali sebesar Rp 450.
-4. [UI] Riwayat mutasi mencatat tipe 'ROLLBACK_REFUND'.</t>
+          <t>1. [API] Webhook endpoint merespons HTTP 200 OK ({"status": "EVENT_RECEIVED"}).
+2. [DB] Status record di broadcast_recipients terupdate menjadi 'FAILED' dengan error code 131026.
+3. [DB] Saldo merchant di wallets bertambah kembali + Rp 750 dengan transaction_type = 'CREDIT_REFUND' dan reference_id = 'wamid.HBgL12345'.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1269,7 +1265,7 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-02: Credit Rollback (Covers: AC-2)</t>
+          <t>[Priority: Critical] US-03: Failed Message Credit Rollback (Covers: AC-1)</t>
         </is>
       </c>
     </row>
@@ -1281,28 +1277,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>DELIVERY_CREDIT</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>JOB-ROLL-RDED-POS-010</t>
+          <t>ROLLBACK_MGMT</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>JOB-ROLL-RD-POS-010</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Resiliency Test: Re-deduct saldo saat webhook Delivered tiba terlambat setelah Rollback</t>
+          <t>Verifikasi status Delivered dari Meta mengunci kredit secara permanen (No Rollback)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Memastikan sistem melakukan pemotongan saldo ulang (re-deduct) jika signal delivered diterima setelah kredit sempat di-rollback</t>
+          <t>Memastikan webhook status 'delivered' dari Meta mengunci pemotongan saldo secara permanen tanpa ada mutasi refund</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>1. Pesan MSG-001 sempat di-rollback karena timeout / initial failure.
-2. Saldo akun mencukupi.</t>
+          <t>1. Pesan MSG-BC-8802 berstatus 'SENT', saldo terpotong Rp 750, wamid = 'wamid.HBgL12346'.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1322,7 +1317,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Resiliency, EdgeCase</t>
+          <t>Webhook, Integration</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -1330,17 +1325,16 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim late webhook 'delivered' untuk MSG-001.
-2. Amati respon webhook handler.
-3. Verifikasi pencatatan transaksi di DB.</t>
+          <t>1. [Arrange] Siapkan payload webhook WhatsApp delivered: {"statuses": [{"id": "wamid.HBgL12346", "status": "delivered", "timestamp": "1726050005"}]}.
+2. [Act] Inject payload webhook ke POST /api/v1/webhooks/whatsapp.
+3. [Assert] Query record broadcast_recipients dan wallet ledger.</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>1. [API] Sistem mendeteksi pesan telah di-rollback sebelumnya.
-2. [DB] Sistem memicu transaksi tipe 'RE_DEDUCTION' sebesar Rp 450.
-3. [DB] Saldo utama terpotong Rp 450 dan status final pesan menjadi 'DELIVERED'.
-4. [UI] Log riwayat kredit mencatat entri re-deduction.</t>
+          <t>1. [API] Webhook merespons HTTP 200 OK.
+2. [DB] Status pesan berubah menjadi 'DELIVERED'.
+3. [DB] Saldo wallet tidak mengalami penambahan refund (refund_amount = 0), dan transaksi terkunci dengan status 'SETTLED'.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1350,7 +1344,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-02: Late Webhook Re-Deduct (Covers: AC-2)</t>
+          <t>[Priority: High] US-03: Delivered Message Credit Settlement (Covers: AC-2)</t>
         </is>
       </c>
     </row>
@@ -1362,37 +1356,37 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>DELIVERY_CREDIT</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CUST-NETT-POS-011</t>
+          <t>ROLLBACK_MGMT</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>API-ROLL-LATE-NEG-011</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi Nett Credit Logging dan ekspor data Credit History</t>
+          <t>Verifikasi webhook status Delivered yang datang setelah refund (Late Webhook Idempotency)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Memastikan perhitungan nett log kredit (temporary deducted - rolled back) akurat dan dapat diekspor di Credit History</t>
+          <t>Memastikan webhook delivered yang tiba terlambat pada pesan yang sudah berstatus FAILED dan telah di-refund tidak menyebabkan pemotongan saldo ganda</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>1. Terdapat 10 pesan: 8 delivered (Rp 3.600) dan 2 failed/rolled back (Rp 900).</t>
+          <t>1. Pesan MSG-BC-8803 sudah berstatus 'FAILED' dan kredit Rp 750 telah di-refund ke merchant 2 jam lalu.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1402,26 +1396,24 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Billing, Export</t>
+          <t>Idempotency, Webhook</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>1. Buka halaman WhatsApp Credit &gt; Credit History.
-2. Periksa ringkasan total deducted.
-3. Klik tombol [Export History].
-4. Unduh dan periksa isi file CSV/Excel.</t>
+          <t>1. [Arrange] Siapkan payload webhook late delivered untuk wamid.HBgL12347 (pesan sudah pernah di-refund).
+2. [Act] Kirim request POST /api/v1/webhooks/whatsapp dengan payload delivered tersebut.
+3. [Assert] Verifikasi idempotency handler pada server log dan DB.</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Tampilan total nett credit deduction = Rp 3.600.
-2. [API] Request export mengembalikan file spreadsheet valid.
-3. [File] Data export memuat baris transaksi lengkap dengan status final (DELIVERED / ROLLED_BACK).
-4. [File] Total nett deduction di file sama persis dengan mutasi database.</t>
+          <t>1. [API] Webhook handler memproses idempotently dan mengembalikan HTTP 200 OK dengan warning log: 'Late delivered event received for already refunded message'.
+2. [DB] Sistem TIDAK melakukan pemotongan saldo ulang (mencegah silent double deduction).
+3. [DB] Saldo merchant tetap utuh dan audit log mencatat anomali late status update.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1431,7 +1423,7 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-02: Nett Credit Logging (Covers: AC-3)</t>
+          <t>[Priority: Normal] US-03: Late Delivery Handling (Covers: AC-3)</t>
         </is>
       </c>
     </row>
@@ -1443,27 +1435,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CREDIT_USAGE</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CUST-MNTH-POS-012</t>
+          <t>ROLLBACK_MGMT</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>JOB-ROLL-RECON-POS-012</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi 'Pengeluaran bulan ini' mencakup biaya Service Message per WABA</t>
+          <t>Verifikasi job rekonsiliasi berkala untuk pesan berstatus menggantung (Stuck in Sent)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Memastikan kartu pengeluaran bulanan pada halaman WhatsApp Credit mengakumulasikan biaya Service Message bersama kategori lain</t>
+          <t>Memastikan background cron job mendeteksi pesan yang menggantung &gt; 24 jam tanpa webhook callback Meta dan melakukan auto-refund</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>1. Pengeluaran Marketing = Rp 50.000, Utility = Rp 20.000, Service Message = Rp 30.000.</t>
+          <t>1. Seed 5 record pesan berstatus 'SENT' dengan sent_at = now() - 25 hours di database.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1483,7 +1475,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>CreditView, UI</t>
+          <t>CronJob, Worker</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1491,16 +1483,16 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>1. Login sebagai Owner / Supervisor.
-2. Buka menu WhatsApp Credit.
-3. Periksa nominal kartu 'Pengeluaran bulan ini' pada nomor WABA terkait.</t>
+          <t>1. [Arrange] Pastikan 5 record pesan menggantung &gt; 24 jam tersedia di tabel broadcast_recipients.
+2. [Act] Trigger cron reconciliation command via CLI: python -m jobs.reconcile_broadcast_status --timeout-hours=24.
+3. [Assert] Evaluasi return code CLI dan state tabel database.</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Kartu 'Pengeluaran bulan ini' menampilkan total Rp 100.000.
-2. [API] Endpoint `/api/v1/waba/monthly-expense` mengembalikan breakdown service_cost = 30000.
-3. [UI] Breakdown per kategori (Marketing, Utility, Auth, Service) tertampil jelas.</t>
+          <t>1. [CLI/JOB] Worker selesai dengan exit code 0 dan output: 'Reconciled 5 stuck messages -&gt; Status updated to TIMEOUT_FAILED, 5 refunds executed'.
+2. [DB] 5 record pesan terupdate statusnya menjadi 'TIMEOUT_FAILED'.
+3. [DB] Saldo merchant ter-refund otomatis sebesar total nilai 5 pesan tersebut di tabel wallet_transactions.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1510,7 +1502,7 @@
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-03: Monthly Expense Service Message (Covers: AC-1)</t>
+          <t>[Priority: High] US-03: Reconciliation Cron Job (Covers: AC-4)</t>
         </is>
       </c>
     </row>
@@ -1522,28 +1514,28 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CREDIT_USAGE</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CUST-LMEX-NEG-013</t>
+          <t>FEP_MGMT</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>WEB-FEP-WIN-POS-013</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi pemblokiran pengiriman pesan saat Monthly Credit Limit tercapai</t>
+          <t>Verifikasi identifikasi jendela 72 jam FEP aktif dan penandaan biaya Rp 0 pada UI Chatroom</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Memastikan sistem mencegah pengiriman pesan berbayar baru dan memunculkan notifikasi limit exhausted saat batas bulanan habis</t>
+          <t>Memastikan chatroom FEP menampilkan visual badge toska [Free Entry Point Active] dan label tarif Rp 0 (Bebas Biaya)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>1. Monthly Credit Limit diset = Rp 100.000.
-2. Akumulasi pengeluaran bulan ini sudah mencapai Rp 100.000.</t>
+          <t>1. Sesi customer dari WhatsApp Ad (CTWA) aktif dengan fep_expires_at = now() + 71 hours.
+2. User login sebagai Agent/Admin.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1553,7 +1545,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1563,7 +1555,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>P1-Core, Limit</t>
+          <t>P1-Core, UI, FEP</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -1571,16 +1563,17 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>1. Buat broadcast baru atau kirim pesan template di chatroom.
-2. Klik tombol kirim.
-3. Amati respon sistem.</t>
+          <t>1. [Given] Sesi FEP aktif untuk chatroom CR-FEP-001 dengan sisa waktu 71 jam.
+2. [When] User membuka direct URL /chatrooms/CR-FEP-001 atau memfilter chat list dengan label 'Free Entry Point'.
+3. [Then] Periksa tampilan visual header chatroom dan input bubble area.</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Muncul alert banner / toast error: 'monthly credit limit has exhausted'.
-2. [API] Request kirim pesan dibatalkan dengan status 422 Unprocessable Entity.
-3. [DB] Tidak ada isolasi kredit yang dieksekusi dan pesan tidak terkirim.</t>
+          <t>1. [Then - UI] Header chatroom menampilkan visual badge toska: [Free Entry Point Active] dengan countdown '71h 58m tersisa'.
+2. [Then - UI] Di atas input box chat tampil label info: 'Tarif Pesan: Rp 0 (Bebas Biaya Meta)'.
+3. [And - API] GET /api/v1/chatrooms/CR-FEP-001 mengembalikan {"fep_active": true, "fep_expires_at": "...", "rate_per_message": 0}.
+4. [And - DB] Kolom fep_session_status pada chat_sessions bernilai 'ACTIVE'.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1590,7 +1583,7 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-03: Monthly Credit Limit Exhausted (Covers: AC-2)</t>
+          <t>[Priority: Critical] US-04: FEP 72-Hour Window &amp; UI Tagging (Covers: AC-1, AC-2)</t>
         </is>
       </c>
     </row>
@@ -1602,32 +1595,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CREDIT_USAGE</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CUST-EXPT-POS-014</t>
+          <t>FEP_MGMT</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>WEB-FEP-SEND-POS-014</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi ekspor Credit History memuat baris Service Message dengan TEMPLATE TYPE='Service'</t>
+          <t>Verifikasi pengiriman pesan dalam jendela FEP tidak memotong saldo kredit merchant</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Memastikan file hasil unduhan riwayat kredit membedakan Service Message dengan template Marketing/Utility/Auth</t>
+          <t>Memastikan pesan teks yang dikirim dalam jendela FEP 72 jam terkirim sukses dengan potongan saldo Rp 0</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>1. Akun telah mengirimkan pesan Service, Marketing, dan Utility.</t>
+          <t>1. Berada di dalam chatroom aktif /chatrooms/CR-FEP-001 dengan saldo wallet Rp 500.000.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1642,24 +1635,26 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Export, CreditHistory</t>
+          <t>P1-Core, Billing, FEP</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>1. Buka menu WhatsApp Credit &gt; Download Usage History.
-2. Pilih periode bulan aktif dan download file.
-3. Buka file hasil ekspor dan filter kolom 'TEMPLATE TYPE'.</t>
+          <t>1. [Given] User berada di chatroom FEP aktif /chatrooms/CR-FEP-001 dengan saldo Rp 500.000.
+2. [When - Step 1] Ketik pesan: 'Halo, terima kasih telah menghubungi kami dari iklan promo!'.
+3. [When - Step 2] Klik tombol kirim [Send] (#btn-send-message).
+4. [Then] Periksa saldo di navbar dan status pesan di bubble chat.</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>1. [File] Terdapat baris data dengan kolom 'TEMPLATE TYPE' = 'Service'.
-2. [File] Kolom biaya per pesan tertera akurat sesuai tarif service message.
-3. [File] Baris service message terbedakan secara jelas dari template Marketing, Utility, dan Authentication.</t>
+          <t>1. [Then - UI] Pesan muncul di bubble chat dengan status checklist delivered.
+2. [Then - UI] Indikator saldo di header navbar TETAP Rp 500.000 (tidak berkurang).
+3. [And - API] POST /api/v1/chatrooms/CR-FEP-001/messages merespons HTTP 200 OK dengan payload {"message_id": "MSG-FEP-101", "deducted_credits": 0, "is_fep": true}.
+4. [And - DB] Record chat_messages tersimpan dengan cost = 0, is_fep = TRUE, dan tidak ada mutasi debit di wallet_transactions.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1669,7 +1664,7 @@
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-03: Credit History Download Service Type (Covers: AC-3)</t>
+          <t>[Priority: Critical] US-04: Zero Deduction in FEP Window (Covers: AC-2)</t>
         </is>
       </c>
     </row>
@@ -1681,28 +1676,28 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-COST-POS-015</t>
+          <t>FEP_MGMT</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>API-FEP-EXP-BVA-015</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi tampilan Ongoing Session Cost real-time pada Chatroom Web</t>
+          <t>Verifikasi Boundary Transisi Kadaluarsa Jendela FEP (Relative Timestamp Seeding)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Memastikan running cost sesi percakapan aktif ter-update secara real-time setiap kali pesan berbayar terkirim</t>
+          <t>Memastikan pesan tepat pada boundary kadaluarsa (now + 1m vs now - 1m) bertransisi dari Rp 0 ke tarif berbayar normal</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>1. Agent membuka room percakapan aktif.
-2. Sesi chatroom baru dimulai (Ongoing Cost = Rp 0).</t>
+          <t>1. Sesi A: FEP aktif dengan fep_expires_at = now() + 1 minute.
+2. Sesi B: FEP expired dengan fep_expires_at = now() - 1 minute.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1712,7 +1707,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1722,26 +1717,24 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Chatroom, RealTime</t>
+          <t>BVA, FEP</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim 1 pesan Service Message (tarif Rp 450).
-2. Amati label 'Biaya Sesi Ini' di header chatroom.
-3. Kirim 1 pesan template Marketing (tarif Rp 600).
-4. Amati perubahan label biaya.</t>
+          <t>1. [Arrange] Setup Sesi A (fep_expires_at = now() + 1m) dan Sesi B (fep_expires_at = now() - 1m) di tabel chat_sessions.
+2. [Act] Kirim pesan ke Sesi A via POST /api/v1/chatrooms/CR-FEP-A/messages dan ke Sesi B via POST /api/v1/chatrooms/CR-FEP-B/messages.
+3. [Assert] Bandingkan deducted_credits pada kedua response API.</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Label biaya sesi langsung berubah menjadi 'Rp 450'.
-2. [UI] Setelah pesan kedua, label biaya ter-update menjadi 'Rp 1.050'.
-3. [API] WebSocket / polling mengembalikan total running cost terkini.
-4. [DB] Record sesi percakapan mencatat running_cost = 1050.</t>
+          <t>1. [API - Sesi A] HTTP 200 OK, deducted_credits = 0, is_fep = true.
+2. [API - Sesi B] HTTP 200 OK, deducted_credits = 300 (tarif normal Service message), is_fep = false.
+3. [DB] Sesi B mencatat mutasi debit Rp 300 di wallet_transactions dan status sesi terupdate menjadi 'EXPIRED'.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1751,7 +1744,7 @@
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-04: Ongoing Session Cost Visibility (Covers: AC-1)</t>
+          <t>[Priority: High] US-04: FEP Expiry Boundary (Covers: AC-3)</t>
         </is>
       </c>
     </row>
@@ -1763,28 +1756,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-FLAT-POS-016</t>
+          <t>FEP_MGMT</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>API-FEP-TEMP-POS-016</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi Owner/Supervisor dapat mengatur Flat Session Limit di Chatroom</t>
+          <t>Verifikasi pengiriman Template Marketing di dalam sesi FEP tetap gratis</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Memastikan konfigurasi flat limit per sesi berlaku universal untuk seluruh percakapan tanpa segmentasi</t>
+          <t>Memastikan template marketing yang dikirimkan ke customer dalam jendela FEP tetap bebas biaya sesuai regulasi Meta</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>1. Login sebagai Owner / Supervisor.
-2. Buka pengaturan limit chatroom.</t>
+          <t>1. Sesi FEP aktif untuk customer 6281234567890.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1804,7 +1796,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Chatroom, Settings</t>
+          <t>FEP, Marketing</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
@@ -1812,16 +1804,15 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>1. Akses setting Flat Session Limit dari quick-access chatroom.
-2. Masukkan limit baru: Rp 10.000.
-3. Klik [Simpan Pengaturan].</t>
+          <t>1. [Arrange] Pastikan customer 6281234567890 terasosiasi dengan sesi FEP aktif.
+2. [Act] Kirim template pesan kategori MARKETING melalui POST /api/v1/messages/send-template.
+3. [Assert] Verifikasi response payload dan persistensi audit billing.</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Muncul toast sukses: 'Pengaturan limit sesi berhasil disimpan'.
-2. [API] Request PUT `/api/v1/chatroom/flat-limit` mengembalikan 200 OK dengan value 10000.
-3. [DB] Seluruh room aktif menerapkan default limit Rp 10.000.</t>
+          <t>1. [API] HTTP 200 OK dengan payload {"status": "SENT", "category": "MARKETING", "billed_cost": 0, "fep_override": true}.
+2. [DB] Record chat_messages mencatat template terkirim dengan cost = 0 dan flag fep_override = TRUE.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1831,7 +1822,7 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-04: Flat Session Limit Setting (Covers: AC-2)</t>
+          <t>[Priority: High] US-04: Marketing Template within FEP (Covers: AC-4)</t>
         </is>
       </c>
     </row>
@@ -1843,38 +1834,38 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-RBAC-SEC-017</t>
+          <t>ALERT_MGMT</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>API-ALRT-DEF-POS-017</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Security Test: Agent tidak memiliki akses untuk mengubah Flat Session Limit utama</t>
+          <t>Verifikasi default threshold batas pengeluaran berlaku untuk seluruh user</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Memastikan role Agent tidak dapat melihat atau mengakses tombol setting Flat Session Limit utama</t>
+          <t>Memastikan konfigurasi default low credit threshold (Rp 50.000) otomatis memicu status low balance pada seluruh akun tanpa konfigurasi custom</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>1. Login sebagai Agent (CS).
-2. Buka dashboard Chatroom Web.</t>
+          <t>1. Konfigurasi DEFAULT_LOW_CREDIT_THRESHOLD = 50000 aktif di DB.
+2. Akun merchant USR-NEW-001 baru terdaftar.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1884,7 +1875,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>RBAC, Security</t>
+          <t>Threshold, Alert</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -1892,16 +1883,15 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>1. Periksa header dan sidebar chatroom untuk menu pengaturan limit.
-2. Coba kirim request PUT `/api/v1/chatroom/flat-limit` via Postman/Direct API.
-3. Amati respon sistem.</t>
+          <t>1. [Arrange] Kurangi saldo USR-NEW-001 hingga bernilai Rp 49.000 (&lt; Rp 50.000).
+2. [Act] Panggil endpoint evaluator threshold POST /api/v1/wallets/check-threshold.
+3. [Assert] Query notifikasi in-app untuk USR-NEW-001.</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Tombol/menu pengaturan Flat Session Limit utama tersembunyi (Hidden).
-2. [API] Direct API call menghasilkan response HTTP 403 Forbidden.
-3. [DB] Nilai flat session limit di database tidak berubah.</t>
+          <t>1. [API] Evaluator merespons {"is_low_balance": true, "threshold_applied": 50000, "current_balance": 49000}.
+2. [DB] Record notifikasi low balance terbentuk di in_app_notifications dengan pesan 'Saldo Anda berada di bawah batas minimum Rp 50.000'.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1911,7 +1901,7 @@
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-04: RBAC Flat Limit Protection (Covers: AC-2)</t>
+          <t>[Priority: High] US-05: Global Default Credit Threshold (Covers: AC-1)</t>
         </is>
       </c>
     </row>
@@ -1923,38 +1913,37 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-BLCK-NEG-018</t>
+          <t>ALERT_MGMT</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>WEB-ALRT-POP-POS-018</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi pemblokiran pengiriman pesan saat Session Cost mencapai limit</t>
+          <t>Verifikasi in-app pop-up / modal warning saat saldo mendekati batas minimum</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Memastikan percakapan diflagged limit-reached dan input chat berbayar disabled saat biaya sesi mencapai limit</t>
+          <t>Memastikan modal dialog peringatan kuning otomatis muncul saat user mengakses dashboard jika saldo &lt; threshold default</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>1. Flat Session Limit = Rp 5.000.
-2. Running cost sesi percakapan sudah mencapai Rp 5.000.</t>
+          <t>1. User login dengan saldo Rp 45.000 (threshold default = Rp 50.000).</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1964,7 +1953,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>P1-Core, LimitReached</t>
+          <t>UI, Alert</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
@@ -1972,17 +1961,17 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>1. Buka room yang telah mencapai limit Rp 5.000.
-2. Periksa status badge di header chatroom.
-3. Coba ketik dan kirim pesan berbayar baru.</t>
+          <t>1. [Given] User memiliki saldo Rp 45.000.
+2. [When] User mengakses halaman /broadcast/list atau /chatrooms.
+3. [Then] Periksa modal pop-up dialog dan navbar badge.</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Muncul banner peringatan: 'Batas limit sesi percakapan telah tercapai'.
-2. [UI] Tombol kirim pesan berbayar berubah menjadi disabled.
-3. [UI] Muncul tombol opsi [+ Tambah Limit Sesi].
-4. [API] Request kirim pesan diblokir dengan status 403 / 422.</t>
+          <t>1. [Then - UI] Muncul modal dialog kuning: 'Peringatan: Saldo Kredit Menipis!' berisi rincian 'Sisa Saldo: Rp 45.000. Segera lakukan top-up agar broadcast tidak terhenti'.
+2. [Then - UI] Terdapat tombol CTA [Top Up Sekarang] dan tombol [Nanti Saja], serta icon saldo di navbar berkedip oranye [Low Balance Warning].
+3. [And - API] GET /api/v1/user/notifications/unread mengembalikan item tipe LOW_BALANCE_ALERT.
+4. [And - DB] Kolom alert_shown_at di user_notification_states terupdate timestamp sekarang.</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -1992,7 +1981,7 @@
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-04: Block Message on Limit Reached (Covers: AC-3)</t>
+          <t>[Priority: High] US-05: Low Balance Modal Trigger (Covers: AC-2)</t>
         </is>
       </c>
     </row>
@@ -2004,33 +1993,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-TPUP-POS-019</t>
+          <t>ALERT_MGMT</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>JOB-ALRT-MAIL-POS-019</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi manual Limit Top-up oleh Agent dengan preset nominal (Rp2k, Rp5k, Rp10k)</t>
+          <t>Verifikasi pengiriman email alert otomatis saat saldo mencapai threshold</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Memastikan Agent dapat menambah limit sesi dengan preset nominal dan membuka blokir kirim pesan</t>
+          <t>Memastikan automated background worker mendeteksi saldo &lt; threshold dan mengirimkan email pemberitahuan ke email merchant</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>1. Percakapan berstatus limit-reached (limit Rp 5.000, cost Rp 5.000).
-2. Saldo utama akun mencukupi.</t>
+          <t>1. Saldo merchant USR-STD-002 (email: merchant@store.com) bernilai Rp 20.000 (&lt; Rp 50.000).</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2045,27 +2033,23 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>P1-Core, TopUp</t>
+          <t>Email, Worker</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>1. Buka dropdown [+ Tambah Limit Sesi].
-2. Pilih preset 'Rp 5.000'.
-3. Klik tombol [Konfirmasi Tambah Limit].
-4. Coba kirim pesan berbayar baru.</t>
+          <t>1. [Arrange] Pastikan merchant USR-STD-002 berstatus low balance dan belum menerima email dalam 24 jam terakhir.
+2. [Act] Eksekusi worker CLI: python -m jobs.send_low_balance_emails.
+3. [Assert] Periksa email queue dan tabel email_logs.</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Limit sesi baru ter-update menjadi Rp 10.000.
-2. [UI] Status banner 'Limit Reached' hilang dan input chat unblocked (aktif kembali).
-3. [API] Endpoint `/api/v1/chatroom/session/top-up` mengembalikan status 200 OK.
-4. [DB] Audit log mencatat: agent_id, room_id, amount=5000, timestamp UTC.
-5. [UI] Pesan baru berhasil terkirim.</t>
+          <t>1. [JOB] Worker selesai dengan 1 email dispatched ke provider SMTP/SendGrid.
+2. [DB] Record tersimpan di tabel email_logs dengan recipient = 'merchant@store.com', subject = 'Peringatan Saldo Everpro Chat Menipis', status = 'SENT'.</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -2075,7 +2059,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] US-04: Manual Session Limit Top-Up (Covers: AC-4)</t>
+          <t>[Priority: Normal] US-05: Automated Email Notification (Covers: AC-3)</t>
         </is>
       </c>
     </row>
@@ -2087,38 +2071,37 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-TPFL-NEG-020</t>
+          <t>ALERT_MGMT</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>WEB-ALRT-DISM-POS-020</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Verifikasi penolakan Top-up saat Saldo Utama WhatsApp Credit akun tidak mencukupi</t>
+          <t>Verifikasi fungsionalitas dismiss alert dan banner reminder persistent</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Memastikan Agent tidak dapat melakukan top-up limit sesi jika saldo utama akun Rp 0 / tidak cukup</t>
+          <t>Memastikan tombol dismiss menutup modal dan mempertahankan banner info kuning di bagian atas halaman tanpa memunculkan modal kembali</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>1. Percakapan berstatus limit-reached.
-2. Saldo utama WhatsApp Credit akun = Rp 1.000.</t>
+          <t>1. Modal dialog low balance sedang terbuka di layar.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -2128,7 +2111,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>TopUp, Negative</t>
+          <t>UI, Alert</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
@@ -2136,17 +2119,16 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>1. Klik [+ Tambah Limit Sesi].
-2. Pilih preset 'Rp 5.000'.
-3. Klik [Konfirmasi Tambah Limit].</t>
+          <t>1. [Given] Modal low balance aktif di layar.
+2. [When] User mengklik tombol [Nanti Saja] (#btn-dismiss-alert) atau ikon close (X).
+3. [Then] Navigasi ke halaman lain dan amati UI.</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Muncul toast error: 'Saldo utama akun tidak mencukupi untuk top-up limit'.
-2. [UI] Limit sesi tidak bertambah dan percakapan tetap diblokir.
-3. [API] Request mengembalikan HTTP 422 Insufficient Balance.
-4. [DB] Tidak ada saldo yang terpotong.</t>
+          <t>1. [Then - UI] Modal dialog tertutup seketika dan tidak muncul kembali saat berpindah rute halaman selama sesi aktif.
+2. [Then - UI] Banner info kuning persistent berukuran ramping tetap menempel di header: '⚠️ Saldo Anda Rp 45.000. Klik di sini untuk Top Up'.
+3. [And - Client] State lowBalanceModalDismissed = true tersimpan di sessionStorage.</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -2156,7 +2138,7 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-04: Top-Up Insufficient Main Balance (Covers: AC-4)</t>
+          <t>[Priority: Low] US-05: Alert Dismissal &amp; Persistent Banner (Covers: AC-4)</t>
         </is>
       </c>
     </row>
@@ -2168,28 +2150,28 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>CHATROOM_LIMIT</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-CONC-CON-021</t>
+          <t>ALERT_MGMT</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>API-ALRT-EDGE-BVA-021</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Concurrency Test: Top-up simultan oleh Agent dan Owner pada room yang sama</t>
+          <t>Verifikasi Boundary Nilai Saldo Tepat pada Threshold (Saldo == 50.000 vs 49.999)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Memastikan sistem memproses kedua mutasi top-up saat Agent dan Owner mengeksekusi top-up di detik yang sama</t>
+          <t>Memastikan batas pemicu alert hanya aktif saat saldo &lt; threshold (&lt; Rp 50.000) dan tidak terpicu saat saldo == Rp 50.000</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>1. Room limit awal = Rp 5.000.
-2. Saldo utama akun mencukupi (Rp 500.000).</t>
+          <t>1. Threshold default = Rp 50.000.
+2. User X saldo = Rp 50.000. User Y saldo = Rp 49.999.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2199,7 +2181,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Concurrency</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2209,7 +2191,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Concurrency, Con</t>
+          <t>BVA, Alert</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
@@ -2217,17 +2199,16 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>1. Agent klik Top-up Rp 5.000 dan Owner klik Top-up Rp 5.000 secara bersamaan (&lt;50ms).
-2. Amati respon sistem pada kedua klien.
-3. Periksa limit akhir pada database.</t>
+          <t>1. [Arrange] Setup User X (saldo 50.000) dan User Y (saldo 49.999).
+2. [Act] Panggil POST /api/v1/wallets/evaluate-threshold untuk kedua user.
+3. [Assert] Bandingkan response payload evaluasi.</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>1. [API] Kedua request top-up diproses sukses (200 OK).
-2. [DB] Total limit sesi bertambah Rp 10.000 (menjadi Rp 15.000).
-3. [DB] Tercatat 2 baris log audit mutasi top-up (satu dari Agent, satu dari Owner).
-4. [UI] Kedua antarmuka ter-sinkronisasi menampilkan limit baru Rp 15.000.</t>
+          <t>1. [API] Response User X: {"alert_triggered": false, "status": "NORMAL"}.
+2. [API] Response User Y: {"alert_triggered": true, "status": "LOW_BALANCE"}.
+3. [DB] Record notifikasi hanya terbentuk untuk User Y di in_app_notifications.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -2237,7 +2218,7 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] US-04: Simultaneous Top-Up Concurrency (Covers: AC-4)</t>
+          <t>[Priority: High] US-05: Exact Threshold Boundary (Covers: AC-5)</t>
         </is>
       </c>
     </row>
@@ -2249,28 +2230,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>EXPLORATORY</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>E2E-BILL-FDEX-EXP-022</t>
+          <t>SECURITY_MGMT</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>API-CONC-RACE-CON-022</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Exploratory Charter: The FedEx Tour (End-to-End Data &amp; Credit Journey)</t>
+          <t>Verifikasi Concurrency &amp; Race Condition saat Eksekusi Simultan Menguras Saldo Terakhir</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Melacak siklus penuh mutasi kredit dari broadcast dispatch, isolasi, webhook failure, rollback, hingga verifikasi data audit export</t>
+          <t>Memastikan isolasi transaksi (ACID) dan database row lock (SELECT FOR UPDATE) mencegah saldo merchant menjadi negatif saat 2 request simultan terjadi</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>1. Akun dengan saldo Rp 50.000.
-2. Broadcast 10 nomor disiapkan.</t>
+          <t>1. User USR-RACE-001 memiliki sisa saldo tepat Rp 750 (hanya cukup 1 pesan).</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2280,7 +2260,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Exploratory</t>
+          <t>Concurrency</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2290,37 +2270,34 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Exploratory, E2E</t>
+          <t>P1-Core, Concurrency</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>1. Trigger broadcast 10 nomor.
-2. Verifikasi isolasi Rp 4.500 di DB.
-3. Simulasikan 5 delivered dan 5 failed dari Meta.
-4. Verifikasi refund Rp 2.250 ke saldo utama.
-5. Download Credit History dan bandingkan baris mutasi.</t>
+          <t>1. [Arrange] Set saldo USR-RACE-001 = Rp 750.
+2. [Act] Tembak 2 request paralel POST /api/v1/broadcasts pada timestamp milidetik yang sama untuk pesan @ Rp 750.
+3. [Assert] Periksa HTTP response dari kedua request dan saldo akhir database.</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>1. [DB] Mutasi isolasi -&gt; deduct -&gt; rollback tercatat konsisten tanpa selisih 1 Rupiah pun.
-2. [UI] Saldo akhir akun = Rp 47.750.
-3. [File] File export memuat 5 status DELIVERED dan 5 status ROLLED_BACK.
-4. [DB] Audit log mencatat seluruh event lifecycle dengan timestamp terurut.</t>
+          <t>1. [API] Request 1 sukses dengan HTTP 201 Created ({"status": "SUCCESS"}).
+2. [API] Request 2 gagal dengan HTTP 422 Unprocessable Entity ({"error": "INSUFFICIENT_CREDITS"}) atau HTTP 409 Conflict.
+3. [DB] Saldo akhir wallet tepat Rp 0 (TIDAK PERNAH bernilai negatif - Rp 750), dan mutasi tercatat tepat 1 baris.</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] Exploratory: The FedEx Credit Tour</t>
+          <t>[Priority: Critical] US-02: Balance Locking &amp; Concurrency (Covers: AC-2, NFR-Integrity)</t>
         </is>
       </c>
     </row>
@@ -2332,37 +2309,37 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>EXPLORATORY</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>WEB-BRD-CHAO-EXP-023</t>
+          <t>SECURITY_MGMT</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>API-SEC-TAMPR-SEC-023</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Exploratory Charter: The Saboteur Tour (Simulasi Network Drop saat Broadcast Trigger)</t>
+          <t>Verifikasi Security &amp; Authorization: Upaya Manipulasi Harga atau IDOR pada Endpoint Broadcast</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Menyelidiki ketahanan sistem saat koneksi jaringan terputus tepat ketika tombol konfirmasi broadcast diklik</t>
+          <t>Memastikan backend menolak manipulasi payload tarif dari client-side dan selalu menghitung biaya dari master database</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>1. Campaign broadcast siap kirim.</t>
+          <t>1. User role Merchant Admin (bukan Biz Ops).</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Exploratory</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2372,35 +2349,33 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Exploratory, Chaos</t>
+          <t>P1-Core, Security, RBAC</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>1. Klik tombol [Kirim Broadcast Sekarang].
-2. Putuskan koneksi jaringan (Airplane Mode) dalam 100ms.
-3. Sambungkan kembali internet setelah 15 detik.
-4. Refresh halaman broadcast dan periksa status campaign.</t>
+          <t>1. [Arrange] Siapkan payload broadcast dengan manipulasi tarif buatan: {"template_id": "TMP-01", "custom_rate": 0, "category": "MARKETING"}.
+2. [Act] Kirim request POST /api/v1/broadcasts dengan payload tersebut.
+3. [Assert] Evaluasi kalkulasi pemotongan saldo pada database.</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Sistem tidak hang / freeze.
-2. [DB] Tidak terjadi duplikasi pengiriman pesan atau duplikasi isolasi kredit.
-3. [UI] Status campaign menampilkan status yang deterministik (antara 'Processing' atau 'Draft').</t>
+          <t>1. [API] Backend mengabaikan field custom_rate client-side atau merespons HTTP 400 Bad Request / 403 Forbidden.
+2. [DB] Sistem tetap menghitung biaya dari master database pricing (Rp 750), saldo terpotong sesuai tarif resmi, dan audit log security mencatat upaya tampering.</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>[Priority: High] Exploratory: The Saboteur Network Chaos Tour</t>
+          <t>[Priority: Critical] US-01 &amp; US-02: Pricing Integrity &amp; RBAC (Covers: NFR-Security)</t>
         </is>
       </c>
     </row>
@@ -2412,33 +2387,33 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>EXPLORATORY</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>WEB-CHAT-RUSH-EXP-024</t>
+          <t>EXPLORATORY_SUITE</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>E2E-EXP-FEDEX-EXP-024</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Exploratory Charter: The Impatient User Tour (Rapid Multiple Top-Up Clicks)</t>
+          <t>Exploratory Charter: The FedEx Tour (Melacak Lifecycle Saldo &amp; Mutasi dari Broadcast hingga Webhook)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Menguji perilaku sistem saat Agent melakukan spamming click tombol top-up dropdown preset secara cepat</t>
+          <t>Menyelidiki integritas penelusuran status pesan dan rekonsiliasi saldo dari 10 pesan dengan variasi respon 8 delivered dan 2 failed</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>1. Room limit-reached.
-2. Saldo utama Rp 20.000.</t>
+          <t>1. Saldo awal merchant Rp 500.000.
+2. Berada di /broadcast/create.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2453,34 +2428,36 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Exploratory, UI-Stress</t>
+          <t>Exploratory, E2E</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>1. Pilih preset Rp 10.000.
-2. Klik tombol [Konfirmasi Tambah Limit] 5 kali berturut-turut dalam 500ms.
-3. Amati limit akhir dan saldo utama.</t>
+          <t>1. [Given] User membuat broadcast 10 nomor (@ Rp 750, total Rp 7.500) dari /broadcast/create.
+2. [When - Step 1] Saldo terpotong Rp 7.500 saat inisiasi.
+3. [When - Step 2] Sistem mengirim pesan ke Meta API.
+4. [When - Step 3] Inject webhook Meta: 8 pesan status 'delivered' dan 2 pesan status 'failed'.
+5. [When - Step 4] User membuka halaman /billing/history dan /broadcast/detail/BRD-FEDEX-01.</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>1. [UI] Tombol langsung disabled setelah klik pertama (Loading state).
-2. [API] Hanya request pertama yang diproses atau request berikutnya terblokir idempotency lock.
-3. [DB] Limit sesi hanya bertambah Rp 10.000 (bukan Rp 50.000) dan saldo utama terpotong tepat Rp 10.000.</t>
+          <t>1. [Then - UI] Halaman detail broadcast menampilkan statistik: Terkirim: 8, Gagal: 2.
+2. [Then - UI] Mutasi saldo di /billing/history menampilkan kredit refund: + Rp 1.500 dengan keterangan 'Refund Broadcast BRD-FEDEX-01'.
+3. [And - DB] Saldo akhir terpotong bersih Rp 6.000 (8 x Rp 750), tabel wallet_transactions memiliki 1 baris debit Rp 7.500 dan 1 baris refund kredit Rp 1.500.</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Normal] Exploratory: The Impatient User Rapid Click Tour</t>
+          <t>[Priority: High] US-02 &amp; US-03: End-to-End Data Lifecycle (Covers: NFR-Reliability)</t>
         </is>
       </c>
     </row>
@@ -2492,32 +2469,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>EXPLORATORY</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>API-CHAT-SECT-EXP-025</t>
+          <t>EXPLORATORY_SUITE</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>E2E-EXP-CHAOS-EXP-025</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Exploratory Charter: The Rogue / Security Tour (Direct Parameter Tampering)</t>
+          <t>Exploratory Charter: The Chaos / Network Drop Tour saat Eksekusi Broadcast Berjalan</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Mencoba membypass limit chatroom dengan memodifikasi payload nominal top-up negatif atau manipulasi room_id milik user lain</t>
+          <t>Menyelidiki ketahanan transaksi saat jaringan terputus tepat ketika request broadcast dikirimkan ke server</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>1. Agent login dan mendapatkan auth token valid.</t>
+          <t>1. Form wizard broadcast 50 kontak siap di-submit.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2532,34 +2509,36 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Exploratory, Security-BOLA</t>
+          <t>Exploratory, Chaos</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>1. Kirim request top-up dengan payload `amount: -5000`.
-2. Kirim request top-up dengan `amount: 999999999` (melebihi saldo).
-3. Kirim request top-up dengan `room_id` yang tidak di-assign ke Agent.</t>
+          <t>1. [Given] User berada pada modal konfirmasi broadcast di /broadcast/create (50 penerima).
+2. [When - Step 1] Klik [Konfirmasi Kirim].
+3. [When - Step 2] Tepat saat spinner berputar (&lt; 100ms), simulasikan pemutusan koneksi internet (Network Offline).
+4. [When - Step 3] Sambungkan kembali internet setelah 15 detik dan refresh halaman (F5).</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>1. [API] Input amount negatif ditolak dengan HTTP 422 Invalid Amount.
-2. [API] Input melebihi saldo ditolak dengan HTTP 422 Insufficient Balance.
-3. [API] Akses ke unassigned room ditolak dengan HTTP 403 Forbidden (BOLA/IDOR protection).</t>
+          <t>1. [Then - UI] Saat offline, muncul toast peringatan: 'Koneksi terputus. Memeriksa status transaksi...'.
+2. [Then - UI] Setelah online dan refresh, halaman /broadcast/list menampilkan status broadcast yang valid ([Processing] / [Completed]), bukan duplicate atau error blank.
+3. [And - API] Idempotency Key pada header X-Idempotency-Key mencegah server memproses request broadcast dua kali.
+4. [And - DB] Saldo wallet hanya dipotong tepat 1 kali untuk 50 pesan.</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>[Priority: Critical] Exploratory: The Rogue Security &amp; BOLA Tour</t>
+          <t>[Priority: Normal] US-02: Network Resilience (Covers: NFR-Resilience)</t>
         </is>
       </c>
     </row>

</xml_diff>